<commit_message>
daily: 收银合规看板 2026-08-06 更新
</commit_message>
<xml_diff>
--- a/cashier/收银合规分析.xlsx
+++ b/cashier/收银合规分析.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>21,079</t>
+          <t>21,076</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19,660</t>
+          <t>19,658</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1,179</t>
+          <t>1,178</t>
         </is>
       </c>
     </row>
@@ -527,108 +527,120 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>剔除笔数（退货订单，不计入）</t>
+          <t>剔除笔数（门店所属分公司标记剔除，不计入）</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1,775</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>剔除笔数（退货订单，不计入）</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1,775</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>规则未覆盖笔数</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>笔数</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>金额(元)</t>
-        </is>
-      </c>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>合规</t>
+          <t>分类</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>19,660</t>
+          <t>笔数</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>72,866,396.21</t>
+          <t>金额(元)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>不合规</t>
+          <t>合规</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>19,658</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1,157,217.46</t>
+          <t>72,865,681.21</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>剔除</t>
+          <t>不合规</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1,179</t>
+          <t>239</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>7,134,904.83</t>
+          <t>1,157,217.46</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>剔除</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1,178</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7,133,530.64</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>规则未覆盖</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>4,499.0</t>
         </is>
@@ -15331,12 +15343,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1,100</t>
+          <t>1,099</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7,068,900.66</t>
+          <t>7,067,526.47</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -15351,7 +15363,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1,100</t>
+          <t>1,099</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -15849,17 +15861,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>82</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>752,383.0</t>
+          <t>752,067.0</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>82</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -16071,17 +16083,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>90,138.0</t>
+          <t>89,739.0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>41</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -16777,7 +16789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F176"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22313,102 +22325,6 @@
       <c r="F173" t="inlineStr">
         <is>
           <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>APR昆明同德广场</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>399.0</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>四川新跃内购店</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>316.0</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>APR昆明七彩云南</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>1,374.19</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -22423,7 +22339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22594,17 +22510,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2,477</t>
+          <t>2,964</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9,947,798.69</t>
+          <t>11,866,078.22</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2,348</t>
+          <t>2,808</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -22614,7 +22530,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>99.66%</t>
+          <t>99.72%</t>
         </is>
       </c>
     </row>
@@ -22647,166 +22563,6 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>99.83%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>（旧）APR成都凯德魅力城</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>145</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>579,700.02</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>139</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>（旧）APR成都环球中心</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>142</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>593,617.72</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>133</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>（旧）APR成都天府环宇坊</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>129</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>452,489.05</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>（旧）APR成都东安天街</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>292,472.74</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>剔除</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2,089.19</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>100.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 收银合规看板 2026-08-06 三列左移(B/C/D)
</commit_message>
<xml_diff>
--- a/cashier/收银合规分析.xlsx
+++ b/cashier/收银合规分析.xlsx
@@ -22350,42 +22350,42 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>合规门店数量</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>不合规门店数量</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>100%合规门店占比</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>笔数</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>金额(元)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>合规</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>不合规</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>分公司合规率</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>合规门店数量</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>不合规门店数量</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>100%合规门店占比</t>
         </is>
       </c>
     </row>
@@ -22397,42 +22397,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>27.0%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>6,473</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>24,971,246.54</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>6,010</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>88</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>98.56%</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>27.0%</t>
         </is>
       </c>
     </row>
@@ -22444,42 +22444,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>29.7%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>5,835</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>24,854,211.39</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>5,351</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>82</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>98.49%</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>29.7%</t>
         </is>
       </c>
     </row>
@@ -22491,42 +22491,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>51.4%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>2,861</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>9,357,404.74</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>2,702</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>98.76%</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>51.4%</t>
         </is>
       </c>
     </row>
@@ -22538,42 +22538,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>47.6%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>1,059</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>3,245,256.34</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>1,004</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>97.67%</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>47.6%</t>
         </is>
       </c>
     </row>
@@ -22585,42 +22585,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>90.0%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>2,964</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>11,866,078.22</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>2,808</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>99.72%</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>90.0%</t>
         </is>
       </c>
     </row>
@@ -22632,42 +22632,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>90.0%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>1,884</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>6,866,731.08</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>1,783</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>99.83%</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>90.0%</t>
         </is>
       </c>
     </row>

</xml_diff>